<commit_message>
Updated missing photos list
</commit_message>
<xml_diff>
--- a/assets/list/graves_missing_photos.xlsx
+++ b/assets/list/graves_missing_photos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1126,13 +1126,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>James Murphy</t>
+          <t>Michael Buckley</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1145,17 +1149,13 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>124</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Michael Buckley</t>
+          <t>Cornelius Coleman</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1163,18 +1163,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>133</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Cornelius Coleman</t>
+          <t>Ellen Noonan</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1182,18 +1182,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ellen Noonan</t>
+          <t>Bartholomew Linehan</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1201,18 +1201,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>140</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>David Barry</t>
+          <t>David Gilsean</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1220,18 +1220,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>137</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bartholomew Linehan</t>
+          <t>Michael Barry</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -1247,10 +1251,14 @@
           <t>140</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>David Gilsean</t>
+          <t>Patrick Hegarty</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1268,12 +1276,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>d</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Michael Barry</t>
+          <t>May Clossey (nee Russell); Christopher Clossey; Ellen (Lena) Clossey</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1291,12 +1299,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>e</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Patrick Hegarty</t>
+          <t>Unknown Unknown</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1314,12 +1322,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>f</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>May Clossey (nee Russell); Christopher Clossey; Ellen (Lena) Clossey</t>
+          <t>Elizabeth Collins</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -1337,12 +1345,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>g</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Unknown Unknown</t>
+          <t>Hanora Collins; Mary Collins</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -1350,22 +1358,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>f</t>
-        </is>
-      </c>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Elizabeth Collins</t>
+          <t>Thomas Coughlan</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -1373,22 +1377,18 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>140</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Hanora Collins; Mary Collins</t>
+          <t>Cornelius Donnell</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -1401,13 +1401,13 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>151</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Thomas Coughlan</t>
+          <t>William Twomey; Thomas Twomey; John Twomey</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -1415,18 +1415,18 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Cornelius Donnell</t>
+          <t>David Dempsey</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -1434,18 +1434,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>144</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>William Twomey; Thomas Twomey; John Twomey</t>
+          <t>Fenaughton</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -1458,13 +1458,13 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>145</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>David Dempsey</t>
+          <t>Mary Fenton</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -1477,13 +1477,13 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>146</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Fenaughton</t>
+          <t>John Fenton</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -1496,13 +1496,13 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>147</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Mary Fenton</t>
+          <t>John Collins; Hanorah Collins; Mary Collins</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -1515,13 +1515,13 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>148</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>John Fenton</t>
+          <t>Patrick Riordan</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -1534,13 +1534,13 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>149</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>John Collins; Hanorah Collins; Mary Collins</t>
+          <t>Evelyn O'Donoghue</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -1553,13 +1553,13 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>150</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Patrick Riordan</t>
+          <t>Unknown Unknown</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -1572,13 +1572,13 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Evelyn O'Donoghue</t>
+          <t>Mary O'Neill</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>153</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -1610,13 +1610,13 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>154</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Mary O'Neill</t>
+          <t>Unknown Unknown</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>156</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>157</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -1700,18 +1700,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>157</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Unknown Unknown</t>
+          <t>Orla Kidney</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -1719,101 +1723,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>169</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Unknown Unknown</t>
+          <t>Owen McAuliffe</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Thomas Collins; Thomas Collins</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>166</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Margaret Mulcahy</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Orla Kidney</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>169</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Owen McAuliffe</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>